<commit_message>
Changes to be committed: 	modified:   README.md 	modified:   app.py 	modified:   data_analysis/uploads/Sample data analysis.xlsx 	modified:   index_docs.py 	modified:   requirements.txt
</commit_message>
<xml_diff>
--- a/data_analysis/uploads/Sample data analysis.xlsx
+++ b/data_analysis/uploads/Sample data analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LocalAiLab\smolagent_rag\old_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934E6BFD-50FC-44C4-8C58-629F7599F5BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F58F84-4F8B-4FF1-BAA3-928D144BA048}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{0267BFEE-83B5-4D8C-991D-7547B863D89A}"/>
   </bookViews>
@@ -30,10 +30,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>salary</t>
+    <t>workhr</t>
   </si>
   <si>
-    <t>workhr</t>
+    <t>monthly salar rate</t>
   </si>
 </sst>
 </file>
@@ -387,13 +387,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBE5F0E8-7AA9-4932-8163-B6A7AD04D6AA}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -443,7 +447,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <f t="shared" ref="A7:A10" si="1">8*20</f>
+        <f t="shared" ref="A7:A9" si="1">8*20</f>
         <v>160</v>
       </c>
       <c r="B7">

</xml_diff>